<commit_message>
docs: tick 27 mục LỆCH của màn Quản lý vụ giải quyết đơn là Đã xong
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SmFzkXpHDf6C7C3AngDcEJ
</commit_message>
<xml_diff>
--- a/docs/DOI-CHIEU-SRS-MOCKUP.xlsx
+++ b/docs/DOI-CHIEU-SRS-MOCKUP.xlsx
@@ -5958,10 +5958,14 @@
       </c>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L105" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="54" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
@@ -6004,10 +6008,14 @@
       </c>
       <c r="K106" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L106" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="54" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
@@ -6050,10 +6058,14 @@
       </c>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L107" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="54" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -6096,10 +6108,14 @@
       </c>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L108" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="54" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
@@ -6142,10 +6158,14 @@
       </c>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L109" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="54" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
@@ -6188,10 +6208,14 @@
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L110" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="54" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
@@ -6234,10 +6258,14 @@
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L111" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="54" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -6280,10 +6308,14 @@
       </c>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L112" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="54" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
@@ -6326,10 +6358,14 @@
       </c>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L113" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="54" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
@@ -6372,10 +6408,14 @@
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L114" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="54" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
@@ -6422,10 +6462,14 @@
       </c>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L115" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="54" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
@@ -6468,10 +6512,14 @@
       </c>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L116" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="54" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
@@ -6514,10 +6562,14 @@
       </c>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L117" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="54" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
@@ -6564,10 +6616,14 @@
       </c>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L118" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="54" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
@@ -6610,10 +6666,14 @@
       </c>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L119" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="54" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
@@ -6656,10 +6716,14 @@
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L120" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="54" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
@@ -6702,10 +6766,14 @@
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L121" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="54" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
@@ -6748,10 +6816,14 @@
       </c>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L122" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="54" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
@@ -6794,10 +6866,14 @@
       </c>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L123" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="54" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
@@ -6840,10 +6916,14 @@
       </c>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L124" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="54" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
@@ -6886,10 +6966,14 @@
       </c>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L125" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="54" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
@@ -6932,10 +7016,14 @@
       </c>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L126" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="54" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
@@ -6978,10 +7066,14 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L127" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="54" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
@@ -7024,10 +7116,14 @@
       </c>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L128" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="54" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
@@ -7074,10 +7170,14 @@
       </c>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L129" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L129" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="54" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
@@ -7124,10 +7224,14 @@
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L130" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="54" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
@@ -7170,10 +7274,14 @@
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L131" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>A1.1 + A1.1b</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="54" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
@@ -33495,12 +33603,12 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Đã xong</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Sửa nhanh, gom được vào ít PR</t>
+          <t>Hoàn tất 27/27 mục LỆCH (A1.1 + A1.1b)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: tick 22 mục THIẾU mức TB/Thấp — hoàn tất màn Quản lý vụ giải quyết đơn (66/295 Lane A)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SmFzkXpHDf6C7C3AngDcEJ
</commit_message>
<xml_diff>
--- a/docs/DOI-CHIEU-SRS-MOCKUP.xlsx
+++ b/docs/DOI-CHIEU-SRS-MOCKUP.xlsx
@@ -3324,10 +3324,14 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L54" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="54" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -3374,10 +3378,14 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L55" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="54" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -3424,10 +3432,14 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L56" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="54" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -3474,10 +3486,14 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="54" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -3524,10 +3540,14 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L58" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="54" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -3574,10 +3594,14 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="54" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -3848,10 +3872,14 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="54" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
@@ -3898,10 +3926,14 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="54" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -3952,10 +3984,14 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="54" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -4002,10 +4038,14 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="54" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -4284,10 +4324,14 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L72" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="54" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -4334,10 +4378,14 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L73" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="54" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -4442,10 +4490,14 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L75" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="54" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -4496,10 +4548,14 @@
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L76" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="54" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -4662,10 +4718,14 @@
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L79" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="54" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -4716,10 +4776,14 @@
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L80" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="54" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -4766,10 +4830,14 @@
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L81" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="54" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -4816,10 +4884,14 @@
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L82" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="54" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
@@ -5090,10 +5162,14 @@
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L87" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="54" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
@@ -5140,10 +5216,14 @@
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="54" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
@@ -5190,10 +5270,14 @@
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L89" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="54" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
@@ -5240,10 +5324,14 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>Chưa xử lý</t>
-        </is>
-      </c>
-      <c r="L90" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>A1.3</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="54" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
@@ -33757,10 +33845,14 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Gộp vào A1.3 (22 mục TB + Thấp)</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="32" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -33796,10 +33888,14 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="inlineStr"/>
+          <t>Đã xong</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Gộp vào A1.3 (22 mục TB + Thấp)</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="32" customHeight="1">
       <c r="A65" s="2" t="inlineStr">

</xml_diff>